<commit_message>
Updated ESP model - 2025-09-13 01:55
</commit_message>
<xml_diff>
--- a/VerveStacks_ESP/BY_Trans.xlsx
+++ b/VerveStacks_ESP/BY_Trans.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{175BD090-9177-48E9-AFCC-2E73ABFECA0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E56CEE1D-1E6F-468E-8EF0-F70318BC75F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28702" yWindow="-98" windowWidth="28995" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="misc." sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="50">
   <si>
     <t>attribute</t>
   </si>
@@ -181,6 +181,9 @@
   </si>
   <si>
     <t>coal,oil</t>
+  </si>
+  <si>
+    <t>-hydro</t>
   </si>
 </sst>
 </file>
@@ -731,6 +734,9 @@
       <c r="C10" t="s">
         <v>38</v>
       </c>
+      <c r="D10" s="3" t="s">
+        <v>49</v>
+      </c>
       <c r="F10" s="3" t="s">
         <v>42</v>
       </c>

</xml_diff>

<commit_message>
Updated ESP model - 2026-04-26 17:45
</commit_message>
<xml_diff>
--- a/VerveStacks_ESP/BY_Trans.xlsx
+++ b/VerveStacks_ESP/BY_Trans.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E56CEE1D-1E6F-468E-8EF0-F70318BC75F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D1EB1B-B45C-4149-AEE2-7B3180C9E8C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="misc." sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="57">
   <si>
     <t>attribute</t>
   </si>
@@ -87,9 +87,6 @@
     <t>*</t>
   </si>
   <si>
-    <t>*[_][_]m</t>
-  </si>
-  <si>
     <t>~TFM_INS</t>
   </si>
   <si>
@@ -147,9 +144,6 @@
     <t>OUT</t>
   </si>
   <si>
-    <t>ep_hydro_ps*</t>
-  </si>
-  <si>
     <t>ELE</t>
   </si>
   <si>
@@ -159,12 +153,6 @@
     <t>life</t>
   </si>
   <si>
-    <t>af</t>
-  </si>
-  <si>
-    <t>-af</t>
-  </si>
-  <si>
     <t>flo_emis</t>
   </si>
   <si>
@@ -184,6 +172,39 @@
   </si>
   <si>
     <t>-hydro</t>
+  </si>
+  <si>
+    <t>hydro</t>
+  </si>
+  <si>
+    <t>start</t>
+  </si>
+  <si>
+    <t>ncap_iled</t>
+  </si>
+  <si>
+    <t>solar</t>
+  </si>
+  <si>
+    <t>windon</t>
+  </si>
+  <si>
+    <t>windoff</t>
+  </si>
+  <si>
+    <t>-ncap_pasti</t>
+  </si>
+  <si>
+    <t>-ncap_af</t>
+  </si>
+  <si>
+    <t>ncap_af</t>
+  </si>
+  <si>
+    <t>ep_m_*</t>
+  </si>
+  <si>
+    <t>*_hydro_ps*</t>
   </si>
 </sst>
 </file>
@@ -596,7 +617,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{982CB9B3-DA63-443B-9AA5-BEE16CBC2D59}">
-  <dimension ref="B3:L12"/>
+  <dimension ref="B3:L25"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9.53125" bestFit="1" customWidth="1"/>
@@ -642,10 +663,10 @@
         <v>13</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.45">
@@ -681,7 +702,7 @@
         <v>8</v>
       </c>
       <c r="E7" t="s">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="G7">
         <v>4</v>
@@ -715,13 +736,16 @@
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>36</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>45</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H9">
         <v>40</v>
@@ -729,59 +753,165 @@
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>38</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>49</v>
+        <v>36</v>
+      </c>
+      <c r="D10" t="s">
+        <v>46</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="H10">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B11" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H11">
         <v>0.9</v>
-      </c>
-    </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B11" t="s">
-        <v>43</v>
-      </c>
-      <c r="D11" t="s">
-        <v>44</v>
-      </c>
-      <c r="E11" t="s">
-        <v>47</v>
-      </c>
-      <c r="H11">
-        <v>0.95</v>
-      </c>
-      <c r="K11" t="s">
-        <v>46</v>
-      </c>
-      <c r="L11" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12" t="s">
         <v>43</v>
       </c>
-      <c r="D12" t="s">
+      <c r="H12">
+        <v>0.95</v>
+      </c>
+      <c r="K12" t="s">
+        <v>42</v>
+      </c>
+      <c r="L12" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13" t="s">
+        <v>43</v>
+      </c>
+      <c r="H13">
+        <v>0.85</v>
+      </c>
+      <c r="K13" t="s">
+        <v>42</v>
+      </c>
+      <c r="L13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" t="s">
+        <v>36</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H14">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="17.649999999999999" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="B20" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B21" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B22" t="s">
         <v>48</v>
       </c>
-      <c r="E12" t="s">
-        <v>47</v>
-      </c>
-      <c r="H12">
-        <v>0.85</v>
-      </c>
-      <c r="K12" t="s">
+      <c r="C22">
+        <v>4</v>
+      </c>
+      <c r="D22" t="s">
         <v>46</v>
       </c>
-      <c r="L12" t="s">
-        <v>45</v>
+      <c r="E22" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B23" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23">
+        <v>1.5</v>
+      </c>
+      <c r="D23" t="s">
+        <v>49</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B24" t="s">
+        <v>48</v>
+      </c>
+      <c r="C24">
+        <v>3</v>
+      </c>
+      <c r="D24" t="s">
+        <v>50</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B25" t="s">
+        <v>48</v>
+      </c>
+      <c r="C25">
+        <v>1.5</v>
+      </c>
+      <c r="D25" t="s">
+        <v>51</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -805,7 +935,7 @@
   <sheetData>
     <row r="3" spans="2:9" ht="17.649999999999999" thickBot="1" x14ac:dyDescent="0.6">
       <c r="B3" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
@@ -813,123 +943,123 @@
         <v>0</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
         <v>24</v>
-      </c>
-      <c r="C5" t="s">
-        <v>25</v>
       </c>
       <c r="E5">
         <v>0.25</v>
       </c>
       <c r="F5" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="I5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
         <v>26</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>27</v>
-      </c>
-      <c r="D6" t="s">
-        <v>28</v>
       </c>
       <c r="E6">
         <v>0.31</v>
       </c>
       <c r="F6" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E7">
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E8">
         <v>0.67</v>
       </c>
       <c r="F8" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E9">
         <v>0.8</v>
       </c>
       <c r="F9" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="I9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" t="s">
         <v>32</v>
-      </c>
-      <c r="C10" t="s">
-        <v>33</v>
       </c>
       <c r="E10">
         <v>1.25</v>
       </c>
       <c r="F10" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="G10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="2:9" ht="17.649999999999999" thickBot="1" x14ac:dyDescent="0.6">
       <c r="B13" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
@@ -937,21 +1067,21 @@
         <v>6</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>